<commit_message>
Gnuplot script and eps file are added
</commit_message>
<xml_diff>
--- a/InitializationResults/WithTrack/Comparison of SPEA2 with SPEA2_SI for each generation (on average).xlsx
+++ b/InitializationResults/WithTrack/Comparison of SPEA2 with SPEA2_SI for each generation (on average).xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="10995" activeTab="4"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="10995" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="EPS" sheetId="1" r:id="rId1"/>
@@ -17,6 +17,7 @@
     <sheet name="HV" sheetId="3" r:id="rId3"/>
     <sheet name="IGD" sheetId="4" r:id="rId4"/>
     <sheet name="Spd" sheetId="5" r:id="rId5"/>
+    <sheet name="Sheet1" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="152511"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="6">
   <si>
     <t>SPEA2</t>
   </si>
@@ -36,214 +37,16 @@
     <t>SPEA2_SI</t>
   </si>
   <si>
-    <t>1 0.657859671844684</t>
+    <t>SPEA2_SI_Eps</t>
   </si>
   <si>
-    <t>2 0.7687851902625128</t>
+    <t>SPEA2_SI_HV</t>
   </si>
   <si>
-    <t>3 0.7958571026972172</t>
+    <t>SPEA2_SI_IGD</t>
   </si>
   <si>
-    <t>4 0.7956027258673871</t>
-  </si>
-  <si>
-    <t>5 0.7903472497039553</t>
-  </si>
-  <si>
-    <t>6 0.8388715828811718</t>
-  </si>
-  <si>
-    <t>7 0.8481279571116311</t>
-  </si>
-  <si>
-    <t>8 0.8576840259744329</t>
-  </si>
-  <si>
-    <t>9 0.848052528681821</t>
-  </si>
-  <si>
-    <t>10 0.8112998193416588</t>
-  </si>
-  <si>
-    <t>11 0.7782125691316707</t>
-  </si>
-  <si>
-    <t>12 0.743891953250883</t>
-  </si>
-  <si>
-    <t>13 0.7264149703654817</t>
-  </si>
-  <si>
-    <t>14 0.7037820249004605</t>
-  </si>
-  <si>
-    <t>15 0.6897710507032292</t>
-  </si>
-  <si>
-    <t>16 0.6792730554997299</t>
-  </si>
-  <si>
-    <t>17 0.6703119256682791</t>
-  </si>
-  <si>
-    <t>18 0.6684944266480952</t>
-  </si>
-  <si>
-    <t>19 0.6644081142905648</t>
-  </si>
-  <si>
-    <t>20 0.6551997404378601</t>
-  </si>
-  <si>
-    <t>21 0.6505898835797393</t>
-  </si>
-  <si>
-    <t>22 0.6521148589876689</t>
-  </si>
-  <si>
-    <t>23 0.643747873115321</t>
-  </si>
-  <si>
-    <t>24 0.6384257353936403</t>
-  </si>
-  <si>
-    <t>25 0.6358761920102745</t>
-  </si>
-  <si>
-    <t>26 0.6254059861687505</t>
-  </si>
-  <si>
-    <t>27 0.6205928112468339</t>
-  </si>
-  <si>
-    <t>28 0.6169665202217068</t>
-  </si>
-  <si>
-    <t>29 0.6186172397165957</t>
-  </si>
-  <si>
-    <t>30 0.6199914964098251</t>
-  </si>
-  <si>
-    <t>31 0.619035319597225</t>
-  </si>
-  <si>
-    <t>32 0.6099213776525532</t>
-  </si>
-  <si>
-    <t>33 0.6067809082383067</t>
-  </si>
-  <si>
-    <t>34 0.6013722844358659</t>
-  </si>
-  <si>
-    <t>35 0.6066667821875183</t>
-  </si>
-  <si>
-    <t>36 0.6017981370478054</t>
-  </si>
-  <si>
-    <t>37 0.5990194350816828</t>
-  </si>
-  <si>
-    <t>38 0.5957329562085255</t>
-  </si>
-  <si>
-    <t>39 0.5945429067610194</t>
-  </si>
-  <si>
-    <t>40 0.5937290987341773</t>
-  </si>
-  <si>
-    <t>41 0.5924686339391932</t>
-  </si>
-  <si>
-    <t>42 0.5919607979306803</t>
-  </si>
-  <si>
-    <t>43 0.5928926922137343</t>
-  </si>
-  <si>
-    <t>44 0.5880168966159321</t>
-  </si>
-  <si>
-    <t>45 0.5861580441523648</t>
-  </si>
-  <si>
-    <t>46 0.5810801535771853</t>
-  </si>
-  <si>
-    <t>47 0.5721780079583937</t>
-  </si>
-  <si>
-    <t>48 0.571335344452591</t>
-  </si>
-  <si>
-    <t>49 0.5683832701954683</t>
-  </si>
-  <si>
-    <t>50 0.5684154366519051</t>
-  </si>
-  <si>
-    <t>51 0.5651624141140955</t>
-  </si>
-  <si>
-    <t>52 0.5624042447506735</t>
-  </si>
-  <si>
-    <t>53 0.5622944549126258</t>
-  </si>
-  <si>
-    <t>54 0.5621040306474071</t>
-  </si>
-  <si>
-    <t>55 0.5632085853123532</t>
-  </si>
-  <si>
-    <t>56 0.5591933793524096</t>
-  </si>
-  <si>
-    <t>57 0.5520190638678893</t>
-  </si>
-  <si>
-    <t>58 0.5518903044392609</t>
-  </si>
-  <si>
-    <t>59 0.5523580829226736</t>
-  </si>
-  <si>
-    <t>60 0.55403685691288</t>
-  </si>
-  <si>
-    <t>61 0.5511270806884873</t>
-  </si>
-  <si>
-    <t>62 0.5493814231779771</t>
-  </si>
-  <si>
-    <t>63 0.54790210541945</t>
-  </si>
-  <si>
-    <t>64 0.5452208153099943</t>
-  </si>
-  <si>
-    <t>65 0.5470420000439783</t>
-  </si>
-  <si>
-    <t>66 0.5504313565799258</t>
-  </si>
-  <si>
-    <t>67 0.549644387141993</t>
-  </si>
-  <si>
-    <t>68 0.547212218559148</t>
-  </si>
-  <si>
-    <t>69 0.5448378494937198</t>
-  </si>
-  <si>
-    <t>70 0.5448378494937198</t>
+    <t>SPEA2_SI_Spd</t>
   </si>
 </sst>
 </file>
@@ -279,9 +82,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1107,11 +913,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="364411552"/>
-        <c:axId val="364411944"/>
+        <c:axId val="117573368"/>
+        <c:axId val="117570232"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="364411552"/>
+        <c:axId val="117573368"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1224,12 +1030,12 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="364411944"/>
+        <c:crossAx val="117570232"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="364411944"/>
+        <c:axId val="117570232"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1286,7 +1092,7 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="364411552"/>
+        <c:crossAx val="117573368"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -2172,11 +1978,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="364413904"/>
-        <c:axId val="364412336"/>
+        <c:axId val="117571016"/>
+        <c:axId val="117571800"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="364413904"/>
+        <c:axId val="117571016"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2289,12 +2095,12 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="364412336"/>
+        <c:crossAx val="117571800"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="364412336"/>
+        <c:axId val="117571800"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2351,7 +2157,7 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="364413904"/>
+        <c:crossAx val="117571016"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -3237,11 +3043,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="364414688"/>
-        <c:axId val="364413512"/>
+        <c:axId val="117572192"/>
+        <c:axId val="117572584"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="364414688"/>
+        <c:axId val="117572192"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3354,12 +3160,12 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="364413512"/>
+        <c:crossAx val="117572584"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="364413512"/>
+        <c:axId val="117572584"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0.65000000000000013"/>
@@ -3417,7 +3223,7 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="364414688"/>
+        <c:crossAx val="117572192"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -4303,11 +4109,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="364415472"/>
-        <c:axId val="364416256"/>
+        <c:axId val="120952184"/>
+        <c:axId val="120951792"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="364415472"/>
+        <c:axId val="120952184"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4420,12 +4226,12 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="364416256"/>
+        <c:crossAx val="120951792"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="364416256"/>
+        <c:axId val="120951792"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4482,7 +4288,7 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="364415472"/>
+        <c:crossAx val="120952184"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -5368,11 +5174,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="364406848"/>
-        <c:axId val="364407240"/>
+        <c:axId val="120957280"/>
+        <c:axId val="120956104"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="364406848"/>
+        <c:axId val="120957280"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5485,12 +5291,12 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="364407240"/>
+        <c:crossAx val="120956104"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="364407240"/>
+        <c:axId val="120956104"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5547,7 +5353,7 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="364406848"/>
+        <c:crossAx val="120957280"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -9565,14 +9371,14 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2" t="s">
+      <c r="B1" s="3"/>
+      <c r="C1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="2"/>
+      <c r="D1" s="3"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2">
@@ -10570,14 +10376,14 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2" t="s">
+      <c r="B1" s="3"/>
+      <c r="C1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="2"/>
+      <c r="D1" s="3"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2">
@@ -11575,14 +11381,14 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2" t="s">
+      <c r="B1" s="3"/>
+      <c r="C1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="2"/>
+      <c r="D1" s="3"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2">
@@ -12580,14 +12386,14 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2" t="s">
+      <c r="B1" s="3"/>
+      <c r="C1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="2"/>
+      <c r="D1" s="3"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2">
@@ -12596,8 +12402,8 @@
       <c r="B2">
         <v>0.26070199936674299</v>
       </c>
-      <c r="C2" t="s">
-        <v>2</v>
+      <c r="C2">
+        <v>1</v>
       </c>
       <c r="D2">
         <v>0.12488100860519601</v>
@@ -12610,8 +12416,8 @@
       <c r="B3">
         <v>0.24569335427127501</v>
       </c>
-      <c r="C3" t="s">
-        <v>3</v>
+      <c r="C3">
+        <v>2</v>
       </c>
       <c r="D3">
         <v>0.114352284307533</v>
@@ -12624,8 +12430,8 @@
       <c r="B4">
         <v>0.21862555087809299</v>
       </c>
-      <c r="C4" t="s">
-        <v>4</v>
+      <c r="C4">
+        <v>3</v>
       </c>
       <c r="D4">
         <v>9.39288119990946E-2</v>
@@ -12638,8 +12444,8 @@
       <c r="B5">
         <v>0.20741124922750201</v>
       </c>
-      <c r="C5" t="s">
-        <v>5</v>
+      <c r="C5">
+        <v>4</v>
       </c>
       <c r="D5">
         <v>8.4781818453746202E-2</v>
@@ -12652,8 +12458,8 @@
       <c r="B6">
         <v>0.199080648969579</v>
       </c>
-      <c r="C6" t="s">
-        <v>6</v>
+      <c r="C6">
+        <v>5</v>
       </c>
       <c r="D6">
         <v>7.2137447445350306E-2</v>
@@ -12666,8 +12472,8 @@
       <c r="B7">
         <v>0.17663795023315901</v>
       </c>
-      <c r="C7" t="s">
-        <v>7</v>
+      <c r="C7">
+        <v>6</v>
       </c>
       <c r="D7">
         <v>6.2838439544546695E-2</v>
@@ -12680,8 +12486,8 @@
       <c r="B8">
         <v>0.176118040566489</v>
       </c>
-      <c r="C8" t="s">
-        <v>8</v>
+      <c r="C8">
+        <v>7</v>
       </c>
       <c r="D8">
         <v>5.5685630485540698E-2</v>
@@ -12694,8 +12500,8 @@
       <c r="B9">
         <v>0.17294063125426301</v>
       </c>
-      <c r="C9" t="s">
-        <v>9</v>
+      <c r="C9">
+        <v>8</v>
       </c>
       <c r="D9">
         <v>5.1725776191935802E-2</v>
@@ -12708,8 +12514,8 @@
       <c r="B10">
         <v>0.17127953041896701</v>
       </c>
-      <c r="C10" t="s">
-        <v>10</v>
+      <c r="C10">
+        <v>9</v>
       </c>
       <c r="D10">
         <v>4.6420094853518098E-2</v>
@@ -12722,8 +12528,8 @@
       <c r="B11">
         <v>0.16703731551889101</v>
       </c>
-      <c r="C11" t="s">
-        <v>11</v>
+      <c r="C11">
+        <v>10</v>
       </c>
       <c r="D11">
         <v>4.2840286682438902E-2</v>
@@ -12736,8 +12542,8 @@
       <c r="B12">
         <v>0.14737615503968399</v>
       </c>
-      <c r="C12" t="s">
-        <v>12</v>
+      <c r="C12">
+        <v>11</v>
       </c>
       <c r="D12">
         <v>4.1567348868420499E-2</v>
@@ -12750,8 +12556,8 @@
       <c r="B13">
         <v>0.139370501662094</v>
       </c>
-      <c r="C13" t="s">
-        <v>13</v>
+      <c r="C13">
+        <v>12</v>
       </c>
       <c r="D13">
         <v>3.95898280000039E-2</v>
@@ -12764,8 +12570,8 @@
       <c r="B14">
         <v>0.134198949147457</v>
       </c>
-      <c r="C14" t="s">
-        <v>14</v>
+      <c r="C14">
+        <v>13</v>
       </c>
       <c r="D14">
         <v>3.8296349145494103E-2</v>
@@ -12778,8 +12584,8 @@
       <c r="B15">
         <v>0.12848419495073399</v>
       </c>
-      <c r="C15" t="s">
-        <v>15</v>
+      <c r="C15">
+        <v>14</v>
       </c>
       <c r="D15">
         <v>3.5921620049663101E-2</v>
@@ -12792,8 +12598,8 @@
       <c r="B16">
         <v>0.124335792509762</v>
       </c>
-      <c r="C16" t="s">
-        <v>16</v>
+      <c r="C16">
+        <v>15</v>
       </c>
       <c r="D16">
         <v>3.5019330534999803E-2</v>
@@ -12806,8 +12612,8 @@
       <c r="B17">
         <v>0.112277800907381</v>
       </c>
-      <c r="C17" t="s">
-        <v>17</v>
+      <c r="C17">
+        <v>16</v>
       </c>
       <c r="D17">
         <v>3.4483123674123102E-2</v>
@@ -12820,8 +12626,8 @@
       <c r="B18">
         <v>0.111203285059739</v>
       </c>
-      <c r="C18" t="s">
-        <v>18</v>
+      <c r="C18">
+        <v>17</v>
       </c>
       <c r="D18">
         <v>3.3479557379548101E-2</v>
@@ -12834,8 +12640,8 @@
       <c r="B19">
         <v>0.10299640475463701</v>
       </c>
-      <c r="C19" t="s">
-        <v>19</v>
+      <c r="C19">
+        <v>18</v>
       </c>
       <c r="D19">
         <v>3.3276569864292102E-2</v>
@@ -12848,8 +12654,8 @@
       <c r="B20">
         <v>0.100019155921117</v>
       </c>
-      <c r="C20" t="s">
-        <v>20</v>
+      <c r="C20">
+        <v>19</v>
       </c>
       <c r="D20">
         <v>3.1870215221005999E-2</v>
@@ -12862,8 +12668,8 @@
       <c r="B21">
         <v>9.7091598652251795E-2</v>
       </c>
-      <c r="C21" t="s">
-        <v>21</v>
+      <c r="C21">
+        <v>20</v>
       </c>
       <c r="D21">
         <v>3.0563786365766701E-2</v>
@@ -12876,8 +12682,8 @@
       <c r="B22">
         <v>9.3586669734792793E-2</v>
       </c>
-      <c r="C22" t="s">
-        <v>22</v>
+      <c r="C22">
+        <v>21</v>
       </c>
       <c r="D22">
         <v>2.9963802381725399E-2</v>
@@ -12890,8 +12696,8 @@
       <c r="B23">
         <v>8.9667037502854E-2</v>
       </c>
-      <c r="C23" t="s">
-        <v>23</v>
+      <c r="C23">
+        <v>22</v>
       </c>
       <c r="D23">
         <v>2.8359916294929399E-2</v>
@@ -12904,8 +12710,8 @@
       <c r="B24">
         <v>8.7411760850928305E-2</v>
       </c>
-      <c r="C24" t="s">
-        <v>24</v>
+      <c r="C24">
+        <v>23</v>
       </c>
       <c r="D24">
         <v>2.8174266071330299E-2</v>
@@ -12918,8 +12724,8 @@
       <c r="B25">
         <v>8.3103209200931602E-2</v>
       </c>
-      <c r="C25" t="s">
-        <v>25</v>
+      <c r="C25">
+        <v>24</v>
       </c>
       <c r="D25">
         <v>2.5930126523408099E-2</v>
@@ -12932,8 +12738,8 @@
       <c r="B26">
         <v>7.5380475411144496E-2</v>
       </c>
-      <c r="C26" t="s">
-        <v>26</v>
+      <c r="C26">
+        <v>25</v>
       </c>
       <c r="D26">
         <v>2.5148921525704301E-2</v>
@@ -12946,8 +12752,8 @@
       <c r="B27">
         <v>7.2831769628116896E-2</v>
       </c>
-      <c r="C27" t="s">
-        <v>27</v>
+      <c r="C27">
+        <v>26</v>
       </c>
       <c r="D27">
         <v>2.43580490858449E-2</v>
@@ -12960,8 +12766,8 @@
       <c r="B28">
         <v>6.9804344280290004E-2</v>
       </c>
-      <c r="C28" t="s">
-        <v>28</v>
+      <c r="C28">
+        <v>27</v>
       </c>
       <c r="D28">
         <v>2.39200192322373E-2</v>
@@ -12974,8 +12780,8 @@
       <c r="B29">
         <v>6.5863900094645794E-2</v>
       </c>
-      <c r="C29" t="s">
-        <v>29</v>
+      <c r="C29">
+        <v>28</v>
       </c>
       <c r="D29">
         <v>2.38549444972334E-2</v>
@@ -12988,8 +12794,8 @@
       <c r="B30">
         <v>6.4905166309931595E-2</v>
       </c>
-      <c r="C30" t="s">
-        <v>30</v>
+      <c r="C30">
+        <v>29</v>
       </c>
       <c r="D30">
         <v>2.19312872326431E-2</v>
@@ -13002,8 +12808,8 @@
       <c r="B31">
         <v>6.3663639343299494E-2</v>
       </c>
-      <c r="C31" t="s">
-        <v>31</v>
+      <c r="C31">
+        <v>30</v>
       </c>
       <c r="D31">
         <v>2.1594455293049802E-2</v>
@@ -13016,8 +12822,8 @@
       <c r="B32">
         <v>6.1062337134811101E-2</v>
       </c>
-      <c r="C32" t="s">
-        <v>32</v>
+      <c r="C32">
+        <v>31</v>
       </c>
       <c r="D32">
         <v>2.10413824630626E-2</v>
@@ -13030,8 +12836,8 @@
       <c r="B33">
         <v>6.0974153083806201E-2</v>
       </c>
-      <c r="C33" t="s">
-        <v>33</v>
+      <c r="C33">
+        <v>32</v>
       </c>
       <c r="D33">
         <v>2.0514102597500399E-2</v>
@@ -13044,8 +12850,8 @@
       <c r="B34">
         <v>5.9697188375601701E-2</v>
       </c>
-      <c r="C34" t="s">
-        <v>34</v>
+      <c r="C34">
+        <v>33</v>
       </c>
       <c r="D34">
         <v>2.02481156285493E-2</v>
@@ -13058,8 +12864,8 @@
       <c r="B35">
         <v>5.8235627647746702E-2</v>
       </c>
-      <c r="C35" t="s">
-        <v>35</v>
+      <c r="C35">
+        <v>34</v>
       </c>
       <c r="D35">
         <v>1.9312676687198899E-2</v>
@@ -13072,8 +12878,8 @@
       <c r="B36">
         <v>5.7523394060693199E-2</v>
       </c>
-      <c r="C36" t="s">
-        <v>36</v>
+      <c r="C36">
+        <v>35</v>
       </c>
       <c r="D36">
         <v>1.90694781455286E-2</v>
@@ -13086,8 +12892,8 @@
       <c r="B37">
         <v>5.3070164930587797E-2</v>
       </c>
-      <c r="C37" t="s">
-        <v>37</v>
+      <c r="C37">
+        <v>36</v>
       </c>
       <c r="D37">
         <v>1.8689364112695499E-2</v>
@@ -13100,8 +12906,8 @@
       <c r="B38">
         <v>5.2148403946328997E-2</v>
       </c>
-      <c r="C38" t="s">
-        <v>38</v>
+      <c r="C38">
+        <v>37</v>
       </c>
       <c r="D38">
         <v>1.7678810341686502E-2</v>
@@ -13114,8 +12920,8 @@
       <c r="B39">
         <v>4.7935878989361698E-2</v>
       </c>
-      <c r="C39" t="s">
-        <v>39</v>
+      <c r="C39">
+        <v>38</v>
       </c>
       <c r="D39">
         <v>1.7586942160676199E-2</v>
@@ -13128,8 +12934,8 @@
       <c r="B40">
         <v>4.5717478012335201E-2</v>
       </c>
-      <c r="C40" t="s">
-        <v>40</v>
+      <c r="C40">
+        <v>39</v>
       </c>
       <c r="D40">
         <v>1.72203223041947E-2</v>
@@ -13142,8 +12948,8 @@
       <c r="B41">
         <v>4.2880229859735101E-2</v>
       </c>
-      <c r="C41" t="s">
-        <v>41</v>
+      <c r="C41">
+        <v>40</v>
       </c>
       <c r="D41">
         <v>1.6482968705710699E-2</v>
@@ -13156,8 +12962,8 @@
       <c r="B42">
         <v>4.23775604470732E-2</v>
       </c>
-      <c r="C42" t="s">
-        <v>42</v>
+      <c r="C42">
+        <v>41</v>
       </c>
       <c r="D42">
         <v>1.5700469331038899E-2</v>
@@ -13170,8 +12976,8 @@
       <c r="B43">
         <v>4.2565971503969298E-2</v>
       </c>
-      <c r="C43" t="s">
-        <v>43</v>
+      <c r="C43">
+        <v>42</v>
       </c>
       <c r="D43">
         <v>1.53200867184663E-2</v>
@@ -13184,8 +12990,8 @@
       <c r="B44">
         <v>4.0802560182957803E-2</v>
       </c>
-      <c r="C44" t="s">
-        <v>44</v>
+      <c r="C44">
+        <v>43</v>
       </c>
       <c r="D44">
         <v>1.4356114620424699E-2</v>
@@ -13198,8 +13004,8 @@
       <c r="B45">
         <v>3.8901584759120603E-2</v>
       </c>
-      <c r="C45" t="s">
-        <v>45</v>
+      <c r="C45">
+        <v>44</v>
       </c>
       <c r="D45">
         <v>1.4019312615009299E-2</v>
@@ -13212,8 +13018,8 @@
       <c r="B46">
         <v>3.7614529315325197E-2</v>
       </c>
-      <c r="C46" t="s">
-        <v>46</v>
+      <c r="C46">
+        <v>45</v>
       </c>
       <c r="D46">
         <v>1.38872225507841E-2</v>
@@ -13226,8 +13032,8 @@
       <c r="B47">
         <v>3.5281791151543902E-2</v>
       </c>
-      <c r="C47" t="s">
-        <v>47</v>
+      <c r="C47">
+        <v>46</v>
       </c>
       <c r="D47">
         <v>1.37061346806392E-2</v>
@@ -13240,8 +13046,8 @@
       <c r="B48">
         <v>3.4466552881035901E-2</v>
       </c>
-      <c r="C48" t="s">
-        <v>48</v>
+      <c r="C48">
+        <v>47</v>
       </c>
       <c r="D48">
         <v>1.3428926441428899E-2</v>
@@ -13254,8 +13060,8 @@
       <c r="B49">
         <v>3.3966376027798603E-2</v>
       </c>
-      <c r="C49" t="s">
-        <v>49</v>
+      <c r="C49">
+        <v>48</v>
       </c>
       <c r="D49">
         <v>1.3172627966171101E-2</v>
@@ -13268,8 +13074,8 @@
       <c r="B50">
         <v>3.2108879977000203E-2</v>
       </c>
-      <c r="C50" t="s">
-        <v>50</v>
+      <c r="C50">
+        <v>49</v>
       </c>
       <c r="D50">
         <v>1.2673635248618901E-2</v>
@@ -13282,8 +13088,8 @@
       <c r="B51">
         <v>3.1206307745831701E-2</v>
       </c>
-      <c r="C51" t="s">
-        <v>51</v>
+      <c r="C51">
+        <v>50</v>
       </c>
       <c r="D51">
         <v>1.2600264350854699E-2</v>
@@ -13296,8 +13102,8 @@
       <c r="B52">
         <v>3.0832354784116899E-2</v>
       </c>
-      <c r="C52" t="s">
-        <v>52</v>
+      <c r="C52">
+        <v>51</v>
       </c>
       <c r="D52">
         <v>1.25343739732538E-2</v>
@@ -13310,8 +13116,8 @@
       <c r="B53">
         <v>2.6932382254637899E-2</v>
       </c>
-      <c r="C53" t="s">
-        <v>53</v>
+      <c r="C53">
+        <v>52</v>
       </c>
       <c r="D53">
         <v>1.24396342929151E-2</v>
@@ -13324,8 +13130,8 @@
       <c r="B54">
         <v>2.6607946964281599E-2</v>
       </c>
-      <c r="C54" t="s">
-        <v>54</v>
+      <c r="C54">
+        <v>53</v>
       </c>
       <c r="D54">
         <v>1.22661371115567E-2</v>
@@ -13338,8 +13144,8 @@
       <c r="B55">
         <v>2.6603271204905601E-2</v>
       </c>
-      <c r="C55" t="s">
-        <v>55</v>
+      <c r="C55">
+        <v>54</v>
       </c>
       <c r="D55">
         <v>1.2211386046059E-2</v>
@@ -13352,8 +13158,8 @@
       <c r="B56">
         <v>2.6353743317352601E-2</v>
       </c>
-      <c r="C56" t="s">
-        <v>56</v>
+      <c r="C56">
+        <v>55</v>
       </c>
       <c r="D56">
         <v>1.22470248796145E-2</v>
@@ -13366,8 +13172,8 @@
       <c r="B57">
         <v>2.58008703583094E-2</v>
       </c>
-      <c r="C57" t="s">
-        <v>57</v>
+      <c r="C57">
+        <v>56</v>
       </c>
       <c r="D57">
         <v>1.19322102775377E-2</v>
@@ -13380,8 +13186,8 @@
       <c r="B58">
         <v>2.3430680760085899E-2</v>
       </c>
-      <c r="C58" t="s">
-        <v>58</v>
+      <c r="C58">
+        <v>57</v>
       </c>
       <c r="D58">
         <v>1.1278553370128E-2</v>
@@ -13394,8 +13200,8 @@
       <c r="B59">
         <v>2.3147045866607499E-2</v>
       </c>
-      <c r="C59" t="s">
-        <v>59</v>
+      <c r="C59">
+        <v>58</v>
       </c>
       <c r="D59">
         <v>1.1234938197526899E-2</v>
@@ -13408,8 +13214,8 @@
       <c r="B60">
         <v>2.2737615191229299E-2</v>
       </c>
-      <c r="C60" t="s">
-        <v>60</v>
+      <c r="C60">
+        <v>59</v>
       </c>
       <c r="D60">
         <v>1.1207669931559E-2</v>
@@ -13422,8 +13228,8 @@
       <c r="B61">
         <v>2.2375714118101901E-2</v>
       </c>
-      <c r="C61" t="s">
-        <v>61</v>
+      <c r="C61">
+        <v>60</v>
       </c>
       <c r="D61">
         <v>1.11214860857934E-2</v>
@@ -13436,8 +13242,8 @@
       <c r="B62">
         <v>2.06754057482436E-2</v>
       </c>
-      <c r="C62" t="s">
-        <v>62</v>
+      <c r="C62">
+        <v>61</v>
       </c>
       <c r="D62">
         <v>1.08408385522512E-2</v>
@@ -13450,8 +13256,8 @@
       <c r="B63">
         <v>2.0422532142128198E-2</v>
       </c>
-      <c r="C63" t="s">
-        <v>63</v>
+      <c r="C63">
+        <v>62</v>
       </c>
       <c r="D63">
         <v>1.0761187520518901E-2</v>
@@ -13464,8 +13270,8 @@
       <c r="B64">
         <v>1.9951577105645699E-2</v>
       </c>
-      <c r="C64" t="s">
-        <v>64</v>
+      <c r="C64">
+        <v>63</v>
       </c>
       <c r="D64">
         <v>1.06864347009179E-2</v>
@@ -13478,8 +13284,8 @@
       <c r="B65">
         <v>1.9839470893254101E-2</v>
       </c>
-      <c r="C65" t="s">
-        <v>65</v>
+      <c r="C65">
+        <v>64</v>
       </c>
       <c r="D65">
         <v>1.0582557118743501E-2</v>
@@ -13492,8 +13298,8 @@
       <c r="B66">
         <v>1.9473258059402001E-2</v>
       </c>
-      <c r="C66" t="s">
-        <v>66</v>
+      <c r="C66">
+        <v>65</v>
       </c>
       <c r="D66">
         <v>1.06353399980451E-2</v>
@@ -13506,8 +13312,8 @@
       <c r="B67">
         <v>1.90500853175011E-2</v>
       </c>
-      <c r="C67" t="s">
-        <v>67</v>
+      <c r="C67">
+        <v>66</v>
       </c>
       <c r="D67">
         <v>1.0642553813495E-2</v>
@@ -13520,8 +13326,8 @@
       <c r="B68">
         <v>1.80244992193348E-2</v>
       </c>
-      <c r="C68" t="s">
-        <v>68</v>
+      <c r="C68">
+        <v>67</v>
       </c>
       <c r="D68">
         <v>1.03163331230575E-2</v>
@@ -13534,8 +13340,8 @@
       <c r="B69">
         <v>1.80719191284298E-2</v>
       </c>
-      <c r="C69" t="s">
-        <v>69</v>
+      <c r="C69">
+        <v>68</v>
       </c>
       <c r="D69">
         <v>1.0170418752764599E-2</v>
@@ -13548,8 +13354,8 @@
       <c r="B70">
         <v>1.7957824332433502E-2</v>
       </c>
-      <c r="C70" t="s">
-        <v>70</v>
+      <c r="C70">
+        <v>69</v>
       </c>
       <c r="D70">
         <v>1.0049070616387001E-2</v>
@@ -13562,8 +13368,8 @@
       <c r="B71">
         <v>1.7957824332433502E-2</v>
       </c>
-      <c r="C71" t="s">
-        <v>71</v>
+      <c r="C71">
+        <v>70</v>
       </c>
       <c r="D71">
         <v>1.0049070616387001E-2</v>
@@ -13585,14 +13391,14 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2" t="s">
+      <c r="B1" s="3"/>
+      <c r="C1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="2"/>
+      <c r="D1" s="3"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2">
@@ -14582,4 +14388,2716 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:L71"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3"/>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" s="3"/>
+      <c r="F1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="H1" s="3"/>
+      <c r="I1" t="s">
+        <v>4</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="K1" s="3"/>
+      <c r="L1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>757.1</v>
+      </c>
+      <c r="C2">
+        <v>366.1</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>0.68884288448075603</v>
+      </c>
+      <c r="F2">
+        <v>0.74643435415784498</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <v>0.26070199936674299</v>
+      </c>
+      <c r="I2">
+        <v>0.12488100860519601</v>
+      </c>
+      <c r="J2">
+        <v>1</v>
+      </c>
+      <c r="K2">
+        <v>0.766327328951392</v>
+      </c>
+      <c r="L2">
+        <v>0.65785967184468397</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>708.93333333333305</v>
+      </c>
+      <c r="C3">
+        <v>335.3</v>
+      </c>
+      <c r="D3">
+        <v>2</v>
+      </c>
+      <c r="E3">
+        <v>0.70314472428445796</v>
+      </c>
+      <c r="F3">
+        <v>0.75931399314186998</v>
+      </c>
+      <c r="G3">
+        <v>2</v>
+      </c>
+      <c r="H3">
+        <v>0.24569335427127501</v>
+      </c>
+      <c r="I3">
+        <v>0.114352284307533</v>
+      </c>
+      <c r="J3">
+        <v>2</v>
+      </c>
+      <c r="K3">
+        <v>0.81028008950052399</v>
+      </c>
+      <c r="L3">
+        <v>0.76878519026251202</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>646.6</v>
+      </c>
+      <c r="C4">
+        <v>278.7</v>
+      </c>
+      <c r="D4">
+        <v>3</v>
+      </c>
+      <c r="E4">
+        <v>0.71986048987838902</v>
+      </c>
+      <c r="F4">
+        <v>0.77501245376561301</v>
+      </c>
+      <c r="G4">
+        <v>3</v>
+      </c>
+      <c r="H4">
+        <v>0.21862555087809299</v>
+      </c>
+      <c r="I4">
+        <v>9.39288119990946E-2</v>
+      </c>
+      <c r="J4">
+        <v>3</v>
+      </c>
+      <c r="K4">
+        <v>0.82334868823943097</v>
+      </c>
+      <c r="L4">
+        <v>0.79585710269721699</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>603.96666666666601</v>
+      </c>
+      <c r="C5">
+        <v>252.933333333333</v>
+      </c>
+      <c r="D5">
+        <v>4</v>
+      </c>
+      <c r="E5">
+        <v>0.73356026085486203</v>
+      </c>
+      <c r="F5">
+        <v>0.78491030668751505</v>
+      </c>
+      <c r="G5">
+        <v>4</v>
+      </c>
+      <c r="H5">
+        <v>0.20741124922750201</v>
+      </c>
+      <c r="I5">
+        <v>8.4781818453746202E-2</v>
+      </c>
+      <c r="J5">
+        <v>4</v>
+      </c>
+      <c r="K5">
+        <v>0.83177270166272699</v>
+      </c>
+      <c r="L5">
+        <v>0.79560272586738701</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>554.93333333333305</v>
+      </c>
+      <c r="C6">
+        <v>226.56666666666601</v>
+      </c>
+      <c r="D6">
+        <v>5</v>
+      </c>
+      <c r="E6">
+        <v>0.74487886485935095</v>
+      </c>
+      <c r="F6">
+        <v>0.79369378338761998</v>
+      </c>
+      <c r="G6">
+        <v>5</v>
+      </c>
+      <c r="H6">
+        <v>0.199080648969579</v>
+      </c>
+      <c r="I6">
+        <v>7.2137447445350306E-2</v>
+      </c>
+      <c r="J6">
+        <v>5</v>
+      </c>
+      <c r="K6">
+        <v>0.83462490203242601</v>
+      </c>
+      <c r="L6">
+        <v>0.79034724970395498</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>503.7</v>
+      </c>
+      <c r="C7">
+        <v>195</v>
+      </c>
+      <c r="D7">
+        <v>6</v>
+      </c>
+      <c r="E7">
+        <v>0.75615098121000901</v>
+      </c>
+      <c r="F7">
+        <v>0.80046780221254299</v>
+      </c>
+      <c r="G7">
+        <v>6</v>
+      </c>
+      <c r="H7">
+        <v>0.17663795023315901</v>
+      </c>
+      <c r="I7">
+        <v>6.2838439544546695E-2</v>
+      </c>
+      <c r="J7">
+        <v>6</v>
+      </c>
+      <c r="K7">
+        <v>0.85029133127237899</v>
+      </c>
+      <c r="L7">
+        <v>0.83887158288117103</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>468.9</v>
+      </c>
+      <c r="C8">
+        <v>166</v>
+      </c>
+      <c r="D8">
+        <v>7</v>
+      </c>
+      <c r="E8">
+        <v>0.76574801368551804</v>
+      </c>
+      <c r="F8">
+        <v>0.80671418660317096</v>
+      </c>
+      <c r="G8">
+        <v>7</v>
+      </c>
+      <c r="H8">
+        <v>0.176118040566489</v>
+      </c>
+      <c r="I8">
+        <v>5.5685630485540698E-2</v>
+      </c>
+      <c r="J8">
+        <v>7</v>
+      </c>
+      <c r="K8">
+        <v>0.85302560474017097</v>
+      </c>
+      <c r="L8">
+        <v>0.84812795711163103</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>452.33333333333297</v>
+      </c>
+      <c r="C9">
+        <v>158.833333333333</v>
+      </c>
+      <c r="D9">
+        <v>8</v>
+      </c>
+      <c r="E9">
+        <v>0.77178283252776803</v>
+      </c>
+      <c r="F9">
+        <v>0.81065807409239399</v>
+      </c>
+      <c r="G9">
+        <v>8</v>
+      </c>
+      <c r="H9">
+        <v>0.17294063125426301</v>
+      </c>
+      <c r="I9">
+        <v>5.1725776191935802E-2</v>
+      </c>
+      <c r="J9">
+        <v>8</v>
+      </c>
+      <c r="K9">
+        <v>0.85489516763487405</v>
+      </c>
+      <c r="L9">
+        <v>0.85768402597443205</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>428.06666666666598</v>
+      </c>
+      <c r="C10">
+        <v>145.9</v>
+      </c>
+      <c r="D10">
+        <v>9</v>
+      </c>
+      <c r="E10">
+        <v>0.77817696783470003</v>
+      </c>
+      <c r="F10">
+        <v>0.81460987400212603</v>
+      </c>
+      <c r="G10">
+        <v>9</v>
+      </c>
+      <c r="H10">
+        <v>0.17127953041896701</v>
+      </c>
+      <c r="I10">
+        <v>4.6420094853518098E-2</v>
+      </c>
+      <c r="J10">
+        <v>9</v>
+      </c>
+      <c r="K10">
+        <v>0.87489784121783898</v>
+      </c>
+      <c r="L10">
+        <v>0.84805252868182102</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>410.3</v>
+      </c>
+      <c r="C11">
+        <v>136.433333333333</v>
+      </c>
+      <c r="D11">
+        <v>10</v>
+      </c>
+      <c r="E11">
+        <v>0.78325327465915395</v>
+      </c>
+      <c r="F11">
+        <v>0.81743322825359399</v>
+      </c>
+      <c r="G11">
+        <v>10</v>
+      </c>
+      <c r="H11">
+        <v>0.16703731551889101</v>
+      </c>
+      <c r="I11">
+        <v>4.2840286682438902E-2</v>
+      </c>
+      <c r="J11">
+        <v>10</v>
+      </c>
+      <c r="K11">
+        <v>0.87315759285928796</v>
+      </c>
+      <c r="L11">
+        <v>0.81129981934165796</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12">
+        <v>371.433333333333</v>
+      </c>
+      <c r="C12">
+        <v>134.13333333333301</v>
+      </c>
+      <c r="D12">
+        <v>11</v>
+      </c>
+      <c r="E12">
+        <v>0.789628746784378</v>
+      </c>
+      <c r="F12">
+        <v>0.81965974495805904</v>
+      </c>
+      <c r="G12">
+        <v>11</v>
+      </c>
+      <c r="H12">
+        <v>0.14737615503968399</v>
+      </c>
+      <c r="I12">
+        <v>4.1567348868420499E-2</v>
+      </c>
+      <c r="J12">
+        <v>11</v>
+      </c>
+      <c r="K12">
+        <v>0.87854885324290199</v>
+      </c>
+      <c r="L12">
+        <v>0.77821256913167003</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13">
+        <v>356.86666666666599</v>
+      </c>
+      <c r="C13">
+        <v>123.766666666666</v>
+      </c>
+      <c r="D13">
+        <v>12</v>
+      </c>
+      <c r="E13">
+        <v>0.79348987699242701</v>
+      </c>
+      <c r="F13">
+        <v>0.82182871758003595</v>
+      </c>
+      <c r="G13">
+        <v>12</v>
+      </c>
+      <c r="H13">
+        <v>0.139370501662094</v>
+      </c>
+      <c r="I13">
+        <v>3.95898280000039E-2</v>
+      </c>
+      <c r="J13">
+        <v>12</v>
+      </c>
+      <c r="K13">
+        <v>0.89383434590856503</v>
+      </c>
+      <c r="L13">
+        <v>0.74389195325088298</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14">
+        <v>342.933333333333</v>
+      </c>
+      <c r="C14">
+        <v>120.06666666666599</v>
+      </c>
+      <c r="D14">
+        <v>13</v>
+      </c>
+      <c r="E14">
+        <v>0.79695635557753997</v>
+      </c>
+      <c r="F14">
+        <v>0.82322835140788697</v>
+      </c>
+      <c r="G14">
+        <v>13</v>
+      </c>
+      <c r="H14">
+        <v>0.134198949147457</v>
+      </c>
+      <c r="I14">
+        <v>3.8296349145494103E-2</v>
+      </c>
+      <c r="J14">
+        <v>13</v>
+      </c>
+      <c r="K14">
+        <v>0.87751344808780096</v>
+      </c>
+      <c r="L14">
+        <v>0.72641497036548097</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15">
+        <v>324.86666666666599</v>
+      </c>
+      <c r="C15">
+        <v>114.833333333333</v>
+      </c>
+      <c r="D15">
+        <v>14</v>
+      </c>
+      <c r="E15">
+        <v>0.80026903103066105</v>
+      </c>
+      <c r="F15">
+        <v>0.82444137961872299</v>
+      </c>
+      <c r="G15">
+        <v>14</v>
+      </c>
+      <c r="H15">
+        <v>0.12848419495073399</v>
+      </c>
+      <c r="I15">
+        <v>3.5921620049663101E-2</v>
+      </c>
+      <c r="J15">
+        <v>14</v>
+      </c>
+      <c r="K15">
+        <v>0.84461262772019896</v>
+      </c>
+      <c r="L15">
+        <v>0.70378202490046005</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16">
+        <v>308.03333333333302</v>
+      </c>
+      <c r="C16">
+        <v>113.266666666666</v>
+      </c>
+      <c r="D16">
+        <v>15</v>
+      </c>
+      <c r="E16">
+        <v>0.803299557952454</v>
+      </c>
+      <c r="F16">
+        <v>0.82533250506185296</v>
+      </c>
+      <c r="G16">
+        <v>15</v>
+      </c>
+      <c r="H16">
+        <v>0.124335792509762</v>
+      </c>
+      <c r="I16">
+        <v>3.5019330534999803E-2</v>
+      </c>
+      <c r="J16">
+        <v>15</v>
+      </c>
+      <c r="K16">
+        <v>0.82511048118899399</v>
+      </c>
+      <c r="L16">
+        <v>0.68977105070322897</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17">
+        <v>279.60000000000002</v>
+      </c>
+      <c r="C17">
+        <v>111.56666666666599</v>
+      </c>
+      <c r="D17">
+        <v>16</v>
+      </c>
+      <c r="E17">
+        <v>0.80729497224190105</v>
+      </c>
+      <c r="F17">
+        <v>0.82594094923894001</v>
+      </c>
+      <c r="G17">
+        <v>16</v>
+      </c>
+      <c r="H17">
+        <v>0.112277800907381</v>
+      </c>
+      <c r="I17">
+        <v>3.4483123674123102E-2</v>
+      </c>
+      <c r="J17">
+        <v>16</v>
+      </c>
+      <c r="K17">
+        <v>0.81221615539852599</v>
+      </c>
+      <c r="L17">
+        <v>0.67927305549972905</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18">
+        <v>275.26666666666603</v>
+      </c>
+      <c r="C18">
+        <v>106.2</v>
+      </c>
+      <c r="D18">
+        <v>17</v>
+      </c>
+      <c r="E18">
+        <v>0.80871178458094495</v>
+      </c>
+      <c r="F18">
+        <v>0.82669980800590204</v>
+      </c>
+      <c r="G18">
+        <v>17</v>
+      </c>
+      <c r="H18">
+        <v>0.111203285059739</v>
+      </c>
+      <c r="I18">
+        <v>3.3479557379548101E-2</v>
+      </c>
+      <c r="J18">
+        <v>17</v>
+      </c>
+      <c r="K18">
+        <v>0.80125635003364204</v>
+      </c>
+      <c r="L18">
+        <v>0.67031192566827902</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19">
+        <v>260.96666666666601</v>
+      </c>
+      <c r="C19">
+        <v>104.333333333333</v>
+      </c>
+      <c r="D19">
+        <v>18</v>
+      </c>
+      <c r="E19">
+        <v>0.81094378583295901</v>
+      </c>
+      <c r="F19">
+        <v>0.82725116223501205</v>
+      </c>
+      <c r="G19">
+        <v>18</v>
+      </c>
+      <c r="H19">
+        <v>0.10299640475463701</v>
+      </c>
+      <c r="I19">
+        <v>3.3276569864292102E-2</v>
+      </c>
+      <c r="J19">
+        <v>18</v>
+      </c>
+      <c r="K19">
+        <v>0.79037244782224803</v>
+      </c>
+      <c r="L19">
+        <v>0.668494426648095</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20">
+        <v>254</v>
+      </c>
+      <c r="C20">
+        <v>101.23333333333299</v>
+      </c>
+      <c r="D20">
+        <v>19</v>
+      </c>
+      <c r="E20">
+        <v>0.81264051969756002</v>
+      </c>
+      <c r="F20">
+        <v>0.82772129625360003</v>
+      </c>
+      <c r="G20">
+        <v>19</v>
+      </c>
+      <c r="H20">
+        <v>0.100019155921117</v>
+      </c>
+      <c r="I20">
+        <v>3.1870215221005999E-2</v>
+      </c>
+      <c r="J20">
+        <v>19</v>
+      </c>
+      <c r="K20">
+        <v>0.77868012774593098</v>
+      </c>
+      <c r="L20">
+        <v>0.66440811429056401</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21">
+        <v>244.166666666666</v>
+      </c>
+      <c r="C21">
+        <v>98.033333333333303</v>
+      </c>
+      <c r="D21">
+        <v>20</v>
+      </c>
+      <c r="E21">
+        <v>0.81417664714586901</v>
+      </c>
+      <c r="F21">
+        <v>0.82829726981318996</v>
+      </c>
+      <c r="G21">
+        <v>20</v>
+      </c>
+      <c r="H21">
+        <v>9.7091598652251795E-2</v>
+      </c>
+      <c r="I21">
+        <v>3.0563786365766701E-2</v>
+      </c>
+      <c r="J21">
+        <v>20</v>
+      </c>
+      <c r="K21">
+        <v>0.76376931486520105</v>
+      </c>
+      <c r="L21">
+        <v>0.65519974043786</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22">
+        <v>236.06666666666601</v>
+      </c>
+      <c r="C22">
+        <v>95.633333333333297</v>
+      </c>
+      <c r="D22">
+        <v>21</v>
+      </c>
+      <c r="E22">
+        <v>0.81553098105630295</v>
+      </c>
+      <c r="F22">
+        <v>0.82874028676149003</v>
+      </c>
+      <c r="G22">
+        <v>21</v>
+      </c>
+      <c r="H22">
+        <v>9.3586669734792793E-2</v>
+      </c>
+      <c r="I22">
+        <v>2.9963802381725399E-2</v>
+      </c>
+      <c r="J22">
+        <v>21</v>
+      </c>
+      <c r="K22">
+        <v>0.75265977772009596</v>
+      </c>
+      <c r="L22">
+        <v>0.65058988357973901</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23">
+        <v>226.73333333333301</v>
+      </c>
+      <c r="C23">
+        <v>91.966666666666598</v>
+      </c>
+      <c r="D23">
+        <v>22</v>
+      </c>
+      <c r="E23">
+        <v>0.81682080166618398</v>
+      </c>
+      <c r="F23">
+        <v>0.82912818750026196</v>
+      </c>
+      <c r="G23">
+        <v>22</v>
+      </c>
+      <c r="H23">
+        <v>8.9667037502854E-2</v>
+      </c>
+      <c r="I23">
+        <v>2.8359916294929399E-2</v>
+      </c>
+      <c r="J23">
+        <v>22</v>
+      </c>
+      <c r="K23">
+        <v>0.73639902090263898</v>
+      </c>
+      <c r="L23">
+        <v>0.65211485898766797</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24">
+        <v>221.1</v>
+      </c>
+      <c r="C24">
+        <v>90.3333333333333</v>
+      </c>
+      <c r="D24">
+        <v>23</v>
+      </c>
+      <c r="E24">
+        <v>0.81811677929202498</v>
+      </c>
+      <c r="F24">
+        <v>0.82951138096016597</v>
+      </c>
+      <c r="G24">
+        <v>23</v>
+      </c>
+      <c r="H24">
+        <v>8.7411760850928305E-2</v>
+      </c>
+      <c r="I24">
+        <v>2.8174266071330299E-2</v>
+      </c>
+      <c r="J24">
+        <v>23</v>
+      </c>
+      <c r="K24">
+        <v>0.72735402655937997</v>
+      </c>
+      <c r="L24">
+        <v>0.643747873115321</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25">
+        <v>212.766666666666</v>
+      </c>
+      <c r="C25">
+        <v>83.433333333333294</v>
+      </c>
+      <c r="D25">
+        <v>24</v>
+      </c>
+      <c r="E25">
+        <v>0.819071745567297</v>
+      </c>
+      <c r="F25">
+        <v>0.82998467645361496</v>
+      </c>
+      <c r="G25">
+        <v>24</v>
+      </c>
+      <c r="H25">
+        <v>8.3103209200931602E-2</v>
+      </c>
+      <c r="I25">
+        <v>2.5930126523408099E-2</v>
+      </c>
+      <c r="J25">
+        <v>24</v>
+      </c>
+      <c r="K25">
+        <v>0.72298202648197096</v>
+      </c>
+      <c r="L25">
+        <v>0.63842573539364</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26">
+        <v>199.2</v>
+      </c>
+      <c r="C26">
+        <v>81.066666666666606</v>
+      </c>
+      <c r="D26">
+        <v>25</v>
+      </c>
+      <c r="E26">
+        <v>0.82057292212501398</v>
+      </c>
+      <c r="F26">
+        <v>0.83030682375528697</v>
+      </c>
+      <c r="G26">
+        <v>25</v>
+      </c>
+      <c r="H26">
+        <v>7.5380475411144496E-2</v>
+      </c>
+      <c r="I26">
+        <v>2.5148921525704301E-2</v>
+      </c>
+      <c r="J26">
+        <v>25</v>
+      </c>
+      <c r="K26">
+        <v>0.72048916237364102</v>
+      </c>
+      <c r="L26">
+        <v>0.63587619201027401</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27">
+        <v>195.7</v>
+      </c>
+      <c r="C27">
+        <v>79.400000000000006</v>
+      </c>
+      <c r="D27">
+        <v>26</v>
+      </c>
+      <c r="E27">
+        <v>0.82133555370175504</v>
+      </c>
+      <c r="F27">
+        <v>0.83061500642076302</v>
+      </c>
+      <c r="G27">
+        <v>26</v>
+      </c>
+      <c r="H27">
+        <v>7.2831769628116896E-2</v>
+      </c>
+      <c r="I27">
+        <v>2.43580490858449E-2</v>
+      </c>
+      <c r="J27">
+        <v>26</v>
+      </c>
+      <c r="K27">
+        <v>0.71743209919367501</v>
+      </c>
+      <c r="L27">
+        <v>0.62540598616874998</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28">
+        <v>187.06666666666601</v>
+      </c>
+      <c r="C28">
+        <v>78</v>
+      </c>
+      <c r="D28">
+        <v>27</v>
+      </c>
+      <c r="E28">
+        <v>0.82206040478056897</v>
+      </c>
+      <c r="F28">
+        <v>0.83086354026496301</v>
+      </c>
+      <c r="G28">
+        <v>27</v>
+      </c>
+      <c r="H28">
+        <v>6.9804344280290004E-2</v>
+      </c>
+      <c r="I28">
+        <v>2.39200192322373E-2</v>
+      </c>
+      <c r="J28">
+        <v>27</v>
+      </c>
+      <c r="K28">
+        <v>0.71099587521481999</v>
+      </c>
+      <c r="L28">
+        <v>0.62059281124683296</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29">
+        <v>178.5</v>
+      </c>
+      <c r="C29">
+        <v>77.566666666666606</v>
+      </c>
+      <c r="D29">
+        <v>28</v>
+      </c>
+      <c r="E29">
+        <v>0.82307323827250001</v>
+      </c>
+      <c r="F29">
+        <v>0.83104494080182001</v>
+      </c>
+      <c r="G29">
+        <v>28</v>
+      </c>
+      <c r="H29">
+        <v>6.5863900094645794E-2</v>
+      </c>
+      <c r="I29">
+        <v>2.38549444972334E-2</v>
+      </c>
+      <c r="J29">
+        <v>28</v>
+      </c>
+      <c r="K29">
+        <v>0.70323181416706104</v>
+      </c>
+      <c r="L29">
+        <v>0.61696652022170595</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30">
+        <v>176.56666666666601</v>
+      </c>
+      <c r="C30">
+        <v>73.433333333333294</v>
+      </c>
+      <c r="D30">
+        <v>29</v>
+      </c>
+      <c r="E30">
+        <v>0.82339367383640205</v>
+      </c>
+      <c r="F30">
+        <v>0.83136824963983602</v>
+      </c>
+      <c r="G30">
+        <v>29</v>
+      </c>
+      <c r="H30">
+        <v>6.4905166309931595E-2</v>
+      </c>
+      <c r="I30">
+        <v>2.19312872326431E-2</v>
+      </c>
+      <c r="J30">
+        <v>29</v>
+      </c>
+      <c r="K30">
+        <v>0.69503470929871403</v>
+      </c>
+      <c r="L30">
+        <v>0.61861723971659499</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31">
+        <v>174.23333333333301</v>
+      </c>
+      <c r="C31">
+        <v>72.233333333333306</v>
+      </c>
+      <c r="D31">
+        <v>30</v>
+      </c>
+      <c r="E31">
+        <v>0.82387204340966902</v>
+      </c>
+      <c r="F31">
+        <v>0.83157100323204003</v>
+      </c>
+      <c r="G31">
+        <v>30</v>
+      </c>
+      <c r="H31">
+        <v>6.3663639343299494E-2</v>
+      </c>
+      <c r="I31">
+        <v>2.1594455293049802E-2</v>
+      </c>
+      <c r="J31">
+        <v>30</v>
+      </c>
+      <c r="K31">
+        <v>0.68906973129747895</v>
+      </c>
+      <c r="L31">
+        <v>0.61999149640982498</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32">
+        <v>166.63333333333301</v>
+      </c>
+      <c r="C32">
+        <v>70.400000000000006</v>
+      </c>
+      <c r="D32">
+        <v>31</v>
+      </c>
+      <c r="E32">
+        <v>0.82464370527648401</v>
+      </c>
+      <c r="F32">
+        <v>0.83179488281233604</v>
+      </c>
+      <c r="G32">
+        <v>31</v>
+      </c>
+      <c r="H32">
+        <v>6.1062337134811101E-2</v>
+      </c>
+      <c r="I32">
+        <v>2.10413824630626E-2</v>
+      </c>
+      <c r="J32">
+        <v>31</v>
+      </c>
+      <c r="K32">
+        <v>0.68477729271847698</v>
+      </c>
+      <c r="L32">
+        <v>0.61903531959722502</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33">
+        <v>166.433333333333</v>
+      </c>
+      <c r="C33">
+        <v>68.566666666666606</v>
+      </c>
+      <c r="D33">
+        <v>32</v>
+      </c>
+      <c r="E33">
+        <v>0.82487748848245002</v>
+      </c>
+      <c r="F33">
+        <v>0.83195484296028599</v>
+      </c>
+      <c r="G33">
+        <v>32</v>
+      </c>
+      <c r="H33">
+        <v>6.0974153083806201E-2</v>
+      </c>
+      <c r="I33">
+        <v>2.0514102597500399E-2</v>
+      </c>
+      <c r="J33">
+        <v>32</v>
+      </c>
+      <c r="K33">
+        <v>0.67884544887061504</v>
+      </c>
+      <c r="L33">
+        <v>0.60992137765255305</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34">
+        <v>163.266666666666</v>
+      </c>
+      <c r="C34">
+        <v>67.5</v>
+      </c>
+      <c r="D34">
+        <v>33</v>
+      </c>
+      <c r="E34">
+        <v>0.82528001759247205</v>
+      </c>
+      <c r="F34">
+        <v>0.83210599115206196</v>
+      </c>
+      <c r="G34">
+        <v>33</v>
+      </c>
+      <c r="H34">
+        <v>5.9697188375601701E-2</v>
+      </c>
+      <c r="I34">
+        <v>2.02481156285493E-2</v>
+      </c>
+      <c r="J34">
+        <v>33</v>
+      </c>
+      <c r="K34">
+        <v>0.67226918092824095</v>
+      </c>
+      <c r="L34">
+        <v>0.60678090823830599</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35">
+        <v>159.86666666666599</v>
+      </c>
+      <c r="C35">
+        <v>64.400000000000006</v>
+      </c>
+      <c r="D35">
+        <v>34</v>
+      </c>
+      <c r="E35">
+        <v>0.82580955589836902</v>
+      </c>
+      <c r="F35">
+        <v>0.83229159243313999</v>
+      </c>
+      <c r="G35">
+        <v>34</v>
+      </c>
+      <c r="H35">
+        <v>5.8235627647746702E-2</v>
+      </c>
+      <c r="I35">
+        <v>1.9312676687198899E-2</v>
+      </c>
+      <c r="J35">
+        <v>34</v>
+      </c>
+      <c r="K35">
+        <v>0.66651065380779495</v>
+      </c>
+      <c r="L35">
+        <v>0.60137228443586499</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36">
+        <v>156.9</v>
+      </c>
+      <c r="C36">
+        <v>63.2</v>
+      </c>
+      <c r="D36">
+        <v>35</v>
+      </c>
+      <c r="E36">
+        <v>0.82609773044531698</v>
+      </c>
+      <c r="F36">
+        <v>0.83238044559678204</v>
+      </c>
+      <c r="G36">
+        <v>35</v>
+      </c>
+      <c r="H36">
+        <v>5.7523394060693199E-2</v>
+      </c>
+      <c r="I36">
+        <v>1.90694781455286E-2</v>
+      </c>
+      <c r="J36">
+        <v>35</v>
+      </c>
+      <c r="K36">
+        <v>0.65983022103404199</v>
+      </c>
+      <c r="L36">
+        <v>0.60666678218751802</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37">
+        <v>148.6</v>
+      </c>
+      <c r="C37">
+        <v>60.266666666666602</v>
+      </c>
+      <c r="D37">
+        <v>36</v>
+      </c>
+      <c r="E37">
+        <v>0.826434837985766</v>
+      </c>
+      <c r="F37">
+        <v>0.83254586409221298</v>
+      </c>
+      <c r="G37">
+        <v>36</v>
+      </c>
+      <c r="H37">
+        <v>5.3070164930587797E-2</v>
+      </c>
+      <c r="I37">
+        <v>1.8689364112695499E-2</v>
+      </c>
+      <c r="J37">
+        <v>36</v>
+      </c>
+      <c r="K37">
+        <v>0.65960200845087402</v>
+      </c>
+      <c r="L37">
+        <v>0.60179813704780505</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38">
+        <v>146.86666666666599</v>
+      </c>
+      <c r="C38">
+        <v>57.1666666666666</v>
+      </c>
+      <c r="D38">
+        <v>37</v>
+      </c>
+      <c r="E38">
+        <v>0.82666695312074201</v>
+      </c>
+      <c r="F38">
+        <v>0.83271850507303102</v>
+      </c>
+      <c r="G38">
+        <v>37</v>
+      </c>
+      <c r="H38">
+        <v>5.2148403946328997E-2</v>
+      </c>
+      <c r="I38">
+        <v>1.7678810341686502E-2</v>
+      </c>
+      <c r="J38">
+        <v>37</v>
+      </c>
+      <c r="K38">
+        <v>0.66029389869948496</v>
+      </c>
+      <c r="L38">
+        <v>0.59901943508168198</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>38</v>
+      </c>
+      <c r="B39">
+        <v>138.6</v>
+      </c>
+      <c r="C39">
+        <v>57</v>
+      </c>
+      <c r="D39">
+        <v>38</v>
+      </c>
+      <c r="E39">
+        <v>0.82731439173223598</v>
+      </c>
+      <c r="F39">
+        <v>0.83280352429340199</v>
+      </c>
+      <c r="G39">
+        <v>38</v>
+      </c>
+      <c r="H39">
+        <v>4.7935878989361698E-2</v>
+      </c>
+      <c r="I39">
+        <v>1.7586942160676199E-2</v>
+      </c>
+      <c r="J39">
+        <v>38</v>
+      </c>
+      <c r="K39">
+        <v>0.66043748103364397</v>
+      </c>
+      <c r="L39">
+        <v>0.59573295620852496</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>39</v>
+      </c>
+      <c r="B40">
+        <v>134.03333333333299</v>
+      </c>
+      <c r="C40">
+        <v>55.4</v>
+      </c>
+      <c r="D40">
+        <v>39</v>
+      </c>
+      <c r="E40">
+        <v>0.82782725806158597</v>
+      </c>
+      <c r="F40">
+        <v>0.83294113578342399</v>
+      </c>
+      <c r="G40">
+        <v>39</v>
+      </c>
+      <c r="H40">
+        <v>4.5717478012335201E-2</v>
+      </c>
+      <c r="I40">
+        <v>1.72203223041947E-2</v>
+      </c>
+      <c r="J40">
+        <v>39</v>
+      </c>
+      <c r="K40">
+        <v>0.65410736450821005</v>
+      </c>
+      <c r="L40">
+        <v>0.59454290676101895</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41">
+        <v>127.533333333333</v>
+      </c>
+      <c r="C41">
+        <v>53.366666666666603</v>
+      </c>
+      <c r="D41">
+        <v>40</v>
+      </c>
+      <c r="E41">
+        <v>0.82825522743754898</v>
+      </c>
+      <c r="F41">
+        <v>0.833089436901154</v>
+      </c>
+      <c r="G41">
+        <v>40</v>
+      </c>
+      <c r="H41">
+        <v>4.2880229859735101E-2</v>
+      </c>
+      <c r="I41">
+        <v>1.6482968705710699E-2</v>
+      </c>
+      <c r="J41">
+        <v>40</v>
+      </c>
+      <c r="K41">
+        <v>0.64995627790920696</v>
+      </c>
+      <c r="L41">
+        <v>0.59372909873417701</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A42">
+        <v>41</v>
+      </c>
+      <c r="B42">
+        <v>125.5</v>
+      </c>
+      <c r="C42">
+        <v>50.5</v>
+      </c>
+      <c r="D42">
+        <v>41</v>
+      </c>
+      <c r="E42">
+        <v>0.82855214407382405</v>
+      </c>
+      <c r="F42">
+        <v>0.83321780850055904</v>
+      </c>
+      <c r="G42">
+        <v>41</v>
+      </c>
+      <c r="H42">
+        <v>4.23775604470732E-2</v>
+      </c>
+      <c r="I42">
+        <v>1.5700469331038899E-2</v>
+      </c>
+      <c r="J42">
+        <v>41</v>
+      </c>
+      <c r="K42">
+        <v>0.644044497560191</v>
+      </c>
+      <c r="L42">
+        <v>0.59246863393919302</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A43">
+        <v>42</v>
+      </c>
+      <c r="B43">
+        <v>122.9</v>
+      </c>
+      <c r="C43">
+        <v>49.466666666666598</v>
+      </c>
+      <c r="D43">
+        <v>42</v>
+      </c>
+      <c r="E43">
+        <v>0.82875297632771405</v>
+      </c>
+      <c r="F43">
+        <v>0.83327315177734196</v>
+      </c>
+      <c r="G43">
+        <v>42</v>
+      </c>
+      <c r="H43">
+        <v>4.2565971503969298E-2</v>
+      </c>
+      <c r="I43">
+        <v>1.53200867184663E-2</v>
+      </c>
+      <c r="J43">
+        <v>42</v>
+      </c>
+      <c r="K43">
+        <v>0.640681368796576</v>
+      </c>
+      <c r="L43">
+        <v>0.59196079793068002</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A44">
+        <v>43</v>
+      </c>
+      <c r="B44">
+        <v>115.666666666666</v>
+      </c>
+      <c r="C44">
+        <v>45.733333333333299</v>
+      </c>
+      <c r="D44">
+        <v>43</v>
+      </c>
+      <c r="E44">
+        <v>0.82916370605899203</v>
+      </c>
+      <c r="F44">
+        <v>0.83338489506698099</v>
+      </c>
+      <c r="G44">
+        <v>43</v>
+      </c>
+      <c r="H44">
+        <v>4.0802560182957803E-2</v>
+      </c>
+      <c r="I44">
+        <v>1.4356114620424699E-2</v>
+      </c>
+      <c r="J44">
+        <v>43</v>
+      </c>
+      <c r="K44">
+        <v>0.63750494020191495</v>
+      </c>
+      <c r="L44">
+        <v>0.59289269221373397</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <v>44</v>
+      </c>
+      <c r="B45">
+        <v>108.966666666666</v>
+      </c>
+      <c r="C45">
+        <v>43.966666666666598</v>
+      </c>
+      <c r="D45">
+        <v>44</v>
+      </c>
+      <c r="E45">
+        <v>0.82944491138787702</v>
+      </c>
+      <c r="F45">
+        <v>0.83347724157300995</v>
+      </c>
+      <c r="G45">
+        <v>44</v>
+      </c>
+      <c r="H45">
+        <v>3.8901584759120603E-2</v>
+      </c>
+      <c r="I45">
+        <v>1.4019312615009299E-2</v>
+      </c>
+      <c r="J45">
+        <v>44</v>
+      </c>
+      <c r="K45">
+        <v>0.63198466526347996</v>
+      </c>
+      <c r="L45">
+        <v>0.58801689661593204</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A46">
+        <v>45</v>
+      </c>
+      <c r="B46">
+        <v>106.533333333333</v>
+      </c>
+      <c r="C46">
+        <v>43.733333333333299</v>
+      </c>
+      <c r="D46">
+        <v>45</v>
+      </c>
+      <c r="E46">
+        <v>0.82972256224088103</v>
+      </c>
+      <c r="F46">
+        <v>0.83356081978964403</v>
+      </c>
+      <c r="G46">
+        <v>45</v>
+      </c>
+      <c r="H46">
+        <v>3.7614529315325197E-2</v>
+      </c>
+      <c r="I46">
+        <v>1.38872225507841E-2</v>
+      </c>
+      <c r="J46">
+        <v>45</v>
+      </c>
+      <c r="K46">
+        <v>0.63054092663786498</v>
+      </c>
+      <c r="L46">
+        <v>0.58615804415236406</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A47">
+        <v>46</v>
+      </c>
+      <c r="B47">
+        <v>98</v>
+      </c>
+      <c r="C47">
+        <v>43.133333333333297</v>
+      </c>
+      <c r="D47">
+        <v>46</v>
+      </c>
+      <c r="E47">
+        <v>0.83030089380658301</v>
+      </c>
+      <c r="F47">
+        <v>0.83365713997264002</v>
+      </c>
+      <c r="G47">
+        <v>46</v>
+      </c>
+      <c r="H47">
+        <v>3.5281791151543902E-2</v>
+      </c>
+      <c r="I47">
+        <v>1.37061346806392E-2</v>
+      </c>
+      <c r="J47">
+        <v>46</v>
+      </c>
+      <c r="K47">
+        <v>0.62997831697649098</v>
+      </c>
+      <c r="L47">
+        <v>0.58108015357718501</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A48">
+        <v>47</v>
+      </c>
+      <c r="B48">
+        <v>95.533333333333303</v>
+      </c>
+      <c r="C48">
+        <v>42.1666666666666</v>
+      </c>
+      <c r="D48">
+        <v>47</v>
+      </c>
+      <c r="E48">
+        <v>0.83046756990527404</v>
+      </c>
+      <c r="F48">
+        <v>0.83373079709689202</v>
+      </c>
+      <c r="G48">
+        <v>47</v>
+      </c>
+      <c r="H48">
+        <v>3.4466552881035901E-2</v>
+      </c>
+      <c r="I48">
+        <v>1.3428926441428899E-2</v>
+      </c>
+      <c r="J48">
+        <v>47</v>
+      </c>
+      <c r="K48">
+        <v>0.62615828724044498</v>
+      </c>
+      <c r="L48">
+        <v>0.57217800795839302</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A49">
+        <v>48</v>
+      </c>
+      <c r="B49">
+        <v>94.866666666666603</v>
+      </c>
+      <c r="C49">
+        <v>41.433333333333302</v>
+      </c>
+      <c r="D49">
+        <v>48</v>
+      </c>
+      <c r="E49">
+        <v>0.83060876207124401</v>
+      </c>
+      <c r="F49">
+        <v>0.83379931027447896</v>
+      </c>
+      <c r="G49">
+        <v>48</v>
+      </c>
+      <c r="H49">
+        <v>3.3966376027798603E-2</v>
+      </c>
+      <c r="I49">
+        <v>1.3172627966171101E-2</v>
+      </c>
+      <c r="J49">
+        <v>48</v>
+      </c>
+      <c r="K49">
+        <v>0.62734237468041298</v>
+      </c>
+      <c r="L49">
+        <v>0.57133534445259104</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A50">
+        <v>49</v>
+      </c>
+      <c r="B50">
+        <v>91.133333333333297</v>
+      </c>
+      <c r="C50">
+        <v>40.566666666666599</v>
+      </c>
+      <c r="D50">
+        <v>49</v>
+      </c>
+      <c r="E50">
+        <v>0.83083917420180597</v>
+      </c>
+      <c r="F50">
+        <v>0.83387454813616202</v>
+      </c>
+      <c r="G50">
+        <v>49</v>
+      </c>
+      <c r="H50">
+        <v>3.2108879977000203E-2</v>
+      </c>
+      <c r="I50">
+        <v>1.2673635248618901E-2</v>
+      </c>
+      <c r="J50">
+        <v>49</v>
+      </c>
+      <c r="K50">
+        <v>0.62414815142538005</v>
+      </c>
+      <c r="L50">
+        <v>0.56838327019546797</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A51">
+        <v>50</v>
+      </c>
+      <c r="B51">
+        <v>88.233333333333306</v>
+      </c>
+      <c r="C51">
+        <v>40.5</v>
+      </c>
+      <c r="D51">
+        <v>50</v>
+      </c>
+      <c r="E51">
+        <v>0.83109091318764605</v>
+      </c>
+      <c r="F51">
+        <v>0.83399286764284597</v>
+      </c>
+      <c r="G51">
+        <v>50</v>
+      </c>
+      <c r="H51">
+        <v>3.1206307745831701E-2</v>
+      </c>
+      <c r="I51">
+        <v>1.2600264350854699E-2</v>
+      </c>
+      <c r="J51">
+        <v>50</v>
+      </c>
+      <c r="K51">
+        <v>0.61887902899456004</v>
+      </c>
+      <c r="L51">
+        <v>0.56841543665190497</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A52">
+        <v>51</v>
+      </c>
+      <c r="B52">
+        <v>87</v>
+      </c>
+      <c r="C52">
+        <v>40.299999999999997</v>
+      </c>
+      <c r="D52">
+        <v>51</v>
+      </c>
+      <c r="E52">
+        <v>0.83117102426196199</v>
+      </c>
+      <c r="F52">
+        <v>0.83408932755953602</v>
+      </c>
+      <c r="G52">
+        <v>51</v>
+      </c>
+      <c r="H52">
+        <v>3.0832354784116899E-2</v>
+      </c>
+      <c r="I52">
+        <v>1.25343739732538E-2</v>
+      </c>
+      <c r="J52">
+        <v>51</v>
+      </c>
+      <c r="K52">
+        <v>0.61278252378585596</v>
+      </c>
+      <c r="L52">
+        <v>0.56516241411409496</v>
+      </c>
+    </row>
+    <row r="53" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A53">
+        <v>52</v>
+      </c>
+      <c r="B53">
+        <v>75.5</v>
+      </c>
+      <c r="C53">
+        <v>39.466666666666598</v>
+      </c>
+      <c r="D53">
+        <v>52</v>
+      </c>
+      <c r="E53">
+        <v>0.83154242769130604</v>
+      </c>
+      <c r="F53">
+        <v>0.83415639100003203</v>
+      </c>
+      <c r="G53">
+        <v>52</v>
+      </c>
+      <c r="H53">
+        <v>2.6932382254637899E-2</v>
+      </c>
+      <c r="I53">
+        <v>1.24396342929151E-2</v>
+      </c>
+      <c r="J53">
+        <v>52</v>
+      </c>
+      <c r="K53">
+        <v>0.61126520231954695</v>
+      </c>
+      <c r="L53">
+        <v>0.56240424475067297</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A54">
+        <v>53</v>
+      </c>
+      <c r="B54">
+        <v>74.066666666666606</v>
+      </c>
+      <c r="C54">
+        <v>38.700000000000003</v>
+      </c>
+      <c r="D54">
+        <v>53</v>
+      </c>
+      <c r="E54">
+        <v>0.83161246047283099</v>
+      </c>
+      <c r="F54">
+        <v>0.83416208514812396</v>
+      </c>
+      <c r="G54">
+        <v>53</v>
+      </c>
+      <c r="H54">
+        <v>2.6607946964281599E-2</v>
+      </c>
+      <c r="I54">
+        <v>1.22661371115567E-2</v>
+      </c>
+      <c r="J54">
+        <v>53</v>
+      </c>
+      <c r="K54">
+        <v>0.60928406811964597</v>
+      </c>
+      <c r="L54">
+        <v>0.56229445491262497</v>
+      </c>
+    </row>
+    <row r="55" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A55">
+        <v>54</v>
+      </c>
+      <c r="B55">
+        <v>73.7</v>
+      </c>
+      <c r="C55">
+        <v>38.700000000000003</v>
+      </c>
+      <c r="D55">
+        <v>54</v>
+      </c>
+      <c r="E55">
+        <v>0.83168864153695798</v>
+      </c>
+      <c r="F55">
+        <v>0.83422113136783804</v>
+      </c>
+      <c r="G55">
+        <v>54</v>
+      </c>
+      <c r="H55">
+        <v>2.6603271204905601E-2</v>
+      </c>
+      <c r="I55">
+        <v>1.2211386046059E-2</v>
+      </c>
+      <c r="J55">
+        <v>54</v>
+      </c>
+      <c r="K55">
+        <v>0.60615338415291198</v>
+      </c>
+      <c r="L55">
+        <v>0.56210403064740699</v>
+      </c>
+    </row>
+    <row r="56" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A56">
+        <v>55</v>
+      </c>
+      <c r="B56">
+        <v>72.966666666666598</v>
+      </c>
+      <c r="C56">
+        <v>37.933333333333302</v>
+      </c>
+      <c r="D56">
+        <v>55</v>
+      </c>
+      <c r="E56">
+        <v>0.831793153607854</v>
+      </c>
+      <c r="F56">
+        <v>0.83425073744457801</v>
+      </c>
+      <c r="G56">
+        <v>55</v>
+      </c>
+      <c r="H56">
+        <v>2.6353743317352601E-2</v>
+      </c>
+      <c r="I56">
+        <v>1.22470248796145E-2</v>
+      </c>
+      <c r="J56">
+        <v>55</v>
+      </c>
+      <c r="K56">
+        <v>0.60342455516900795</v>
+      </c>
+      <c r="L56">
+        <v>0.56320858531235296</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A57">
+        <v>56</v>
+      </c>
+      <c r="B57">
+        <v>71.733333333333306</v>
+      </c>
+      <c r="C57">
+        <v>36.533333333333303</v>
+      </c>
+      <c r="D57">
+        <v>56</v>
+      </c>
+      <c r="E57">
+        <v>0.83189143879594196</v>
+      </c>
+      <c r="F57">
+        <v>0.83431475294383906</v>
+      </c>
+      <c r="G57">
+        <v>56</v>
+      </c>
+      <c r="H57">
+        <v>2.58008703583094E-2</v>
+      </c>
+      <c r="I57">
+        <v>1.19322102775377E-2</v>
+      </c>
+      <c r="J57">
+        <v>56</v>
+      </c>
+      <c r="K57">
+        <v>0.60255006745098805</v>
+      </c>
+      <c r="L57">
+        <v>0.55919337935240898</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A58">
+        <v>57</v>
+      </c>
+      <c r="B58">
+        <v>68.066666666666606</v>
+      </c>
+      <c r="C58">
+        <v>34.3333333333333</v>
+      </c>
+      <c r="D58">
+        <v>57</v>
+      </c>
+      <c r="E58">
+        <v>0.83228256214306695</v>
+      </c>
+      <c r="F58">
+        <v>0.83441267133097696</v>
+      </c>
+      <c r="G58">
+        <v>57</v>
+      </c>
+      <c r="H58">
+        <v>2.3430680760085899E-2</v>
+      </c>
+      <c r="I58">
+        <v>1.1278553370128E-2</v>
+      </c>
+      <c r="J58">
+        <v>57</v>
+      </c>
+      <c r="K58">
+        <v>0.59902987081057002</v>
+      </c>
+      <c r="L58">
+        <v>0.55201906386788901</v>
+      </c>
+    </row>
+    <row r="59" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A59">
+        <v>58</v>
+      </c>
+      <c r="B59">
+        <v>66.266666666666595</v>
+      </c>
+      <c r="C59">
+        <v>33.966666666666598</v>
+      </c>
+      <c r="D59">
+        <v>58</v>
+      </c>
+      <c r="E59">
+        <v>0.83239659357197004</v>
+      </c>
+      <c r="F59">
+        <v>0.83444036480275896</v>
+      </c>
+      <c r="G59">
+        <v>58</v>
+      </c>
+      <c r="H59">
+        <v>2.3147045866607499E-2</v>
+      </c>
+      <c r="I59">
+        <v>1.1234938197526899E-2</v>
+      </c>
+      <c r="J59">
+        <v>58</v>
+      </c>
+      <c r="K59">
+        <v>0.59621234806785195</v>
+      </c>
+      <c r="L59">
+        <v>0.55189030443926002</v>
+      </c>
+    </row>
+    <row r="60" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A60">
+        <v>59</v>
+      </c>
+      <c r="B60">
+        <v>65.266666666666595</v>
+      </c>
+      <c r="C60">
+        <v>33.5</v>
+      </c>
+      <c r="D60">
+        <v>59</v>
+      </c>
+      <c r="E60">
+        <v>0.83247404097271405</v>
+      </c>
+      <c r="F60">
+        <v>0.834482520712027</v>
+      </c>
+      <c r="G60">
+        <v>59</v>
+      </c>
+      <c r="H60">
+        <v>2.2737615191229299E-2</v>
+      </c>
+      <c r="I60">
+        <v>1.1207669931559E-2</v>
+      </c>
+      <c r="J60">
+        <v>59</v>
+      </c>
+      <c r="K60">
+        <v>0.59379821765230101</v>
+      </c>
+      <c r="L60">
+        <v>0.55235808292267297</v>
+      </c>
+    </row>
+    <row r="61" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A61">
+        <v>60</v>
+      </c>
+      <c r="B61">
+        <v>64</v>
+      </c>
+      <c r="C61">
+        <v>32.6666666666666</v>
+      </c>
+      <c r="D61">
+        <v>60</v>
+      </c>
+      <c r="E61">
+        <v>0.83261602787407696</v>
+      </c>
+      <c r="F61">
+        <v>0.83451293899087098</v>
+      </c>
+      <c r="G61">
+        <v>60</v>
+      </c>
+      <c r="H61">
+        <v>2.2375714118101901E-2</v>
+      </c>
+      <c r="I61">
+        <v>1.11214860857934E-2</v>
+      </c>
+      <c r="J61">
+        <v>60</v>
+      </c>
+      <c r="K61">
+        <v>0.590989217035776</v>
+      </c>
+      <c r="L61">
+        <v>0.55403685691287996</v>
+      </c>
+    </row>
+    <row r="62" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A62">
+        <v>61</v>
+      </c>
+      <c r="B62">
+        <v>60.933333333333302</v>
+      </c>
+      <c r="C62">
+        <v>31.1666666666666</v>
+      </c>
+      <c r="D62">
+        <v>61</v>
+      </c>
+      <c r="E62">
+        <v>0.832739168193257</v>
+      </c>
+      <c r="F62">
+        <v>0.83456176718410002</v>
+      </c>
+      <c r="G62">
+        <v>61</v>
+      </c>
+      <c r="H62">
+        <v>2.06754057482436E-2</v>
+      </c>
+      <c r="I62">
+        <v>1.08408385522512E-2</v>
+      </c>
+      <c r="J62">
+        <v>61</v>
+      </c>
+      <c r="K62">
+        <v>0.59087769919958799</v>
+      </c>
+      <c r="L62">
+        <v>0.55112708068848704</v>
+      </c>
+    </row>
+    <row r="63" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A63">
+        <v>62</v>
+      </c>
+      <c r="B63">
+        <v>59.9</v>
+      </c>
+      <c r="C63">
+        <v>30.1</v>
+      </c>
+      <c r="D63">
+        <v>62</v>
+      </c>
+      <c r="E63">
+        <v>0.83275938591232801</v>
+      </c>
+      <c r="F63">
+        <v>0.83457872736139405</v>
+      </c>
+      <c r="G63">
+        <v>62</v>
+      </c>
+      <c r="H63">
+        <v>2.0422532142128198E-2</v>
+      </c>
+      <c r="I63">
+        <v>1.0761187520518901E-2</v>
+      </c>
+      <c r="J63">
+        <v>62</v>
+      </c>
+      <c r="K63">
+        <v>0.58865451722088302</v>
+      </c>
+      <c r="L63">
+        <v>0.549381423177977</v>
+      </c>
+    </row>
+    <row r="64" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A64">
+        <v>63</v>
+      </c>
+      <c r="B64">
+        <v>58</v>
+      </c>
+      <c r="C64">
+        <v>29.8</v>
+      </c>
+      <c r="D64">
+        <v>63</v>
+      </c>
+      <c r="E64">
+        <v>0.832899748409481</v>
+      </c>
+      <c r="F64">
+        <v>0.83461091851150104</v>
+      </c>
+      <c r="G64">
+        <v>63</v>
+      </c>
+      <c r="H64">
+        <v>1.9951577105645699E-2</v>
+      </c>
+      <c r="I64">
+        <v>1.06864347009179E-2</v>
+      </c>
+      <c r="J64">
+        <v>63</v>
+      </c>
+      <c r="K64">
+        <v>0.58208297535624598</v>
+      </c>
+      <c r="L64">
+        <v>0.54790210541944995</v>
+      </c>
+    </row>
+    <row r="65" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A65">
+        <v>64</v>
+      </c>
+      <c r="B65">
+        <v>56.733333333333299</v>
+      </c>
+      <c r="C65">
+        <v>29.3</v>
+      </c>
+      <c r="D65">
+        <v>64</v>
+      </c>
+      <c r="E65">
+        <v>0.83297343173380201</v>
+      </c>
+      <c r="F65">
+        <v>0.83465841050126599</v>
+      </c>
+      <c r="G65">
+        <v>64</v>
+      </c>
+      <c r="H65">
+        <v>1.9839470893254101E-2</v>
+      </c>
+      <c r="I65">
+        <v>1.0582557118743501E-2</v>
+      </c>
+      <c r="J65">
+        <v>64</v>
+      </c>
+      <c r="K65">
+        <v>0.58584005692535002</v>
+      </c>
+      <c r="L65">
+        <v>0.545220815309994</v>
+      </c>
+    </row>
+    <row r="66" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A66">
+        <v>65</v>
+      </c>
+      <c r="B66">
+        <v>55.8333333333333</v>
+      </c>
+      <c r="C66">
+        <v>29.1666666666666</v>
+      </c>
+      <c r="D66">
+        <v>65</v>
+      </c>
+      <c r="E66">
+        <v>0.83307887827378602</v>
+      </c>
+      <c r="F66">
+        <v>0.83467005206477496</v>
+      </c>
+      <c r="G66">
+        <v>65</v>
+      </c>
+      <c r="H66">
+        <v>1.9473258059402001E-2</v>
+      </c>
+      <c r="I66">
+        <v>1.06353399980451E-2</v>
+      </c>
+      <c r="J66">
+        <v>65</v>
+      </c>
+      <c r="K66">
+        <v>0.58307570775395201</v>
+      </c>
+      <c r="L66">
+        <v>0.54704200004397796</v>
+      </c>
+    </row>
+    <row r="67" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A67">
+        <v>66</v>
+      </c>
+      <c r="B67">
+        <v>54.233333333333299</v>
+      </c>
+      <c r="C67">
+        <v>29.066666666666599</v>
+      </c>
+      <c r="D67">
+        <v>66</v>
+      </c>
+      <c r="E67">
+        <v>0.83316967024245103</v>
+      </c>
+      <c r="F67">
+        <v>0.83466167677639902</v>
+      </c>
+      <c r="G67">
+        <v>66</v>
+      </c>
+      <c r="H67">
+        <v>1.90500853175011E-2</v>
+      </c>
+      <c r="I67">
+        <v>1.0642553813495E-2</v>
+      </c>
+      <c r="J67">
+        <v>66</v>
+      </c>
+      <c r="K67">
+        <v>0.57981293783868104</v>
+      </c>
+      <c r="L67">
+        <v>0.55043135657992504</v>
+      </c>
+    </row>
+    <row r="68" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A68">
+        <v>67</v>
+      </c>
+      <c r="B68">
+        <v>50</v>
+      </c>
+      <c r="C68">
+        <v>27.3</v>
+      </c>
+      <c r="D68">
+        <v>67</v>
+      </c>
+      <c r="E68">
+        <v>0.83329008575456898</v>
+      </c>
+      <c r="F68">
+        <v>0.83467927448867896</v>
+      </c>
+      <c r="G68">
+        <v>67</v>
+      </c>
+      <c r="H68">
+        <v>1.80244992193348E-2</v>
+      </c>
+      <c r="I68">
+        <v>1.03163331230575E-2</v>
+      </c>
+      <c r="J68">
+        <v>67</v>
+      </c>
+      <c r="K68">
+        <v>0.57713306137931397</v>
+      </c>
+      <c r="L68">
+        <v>0.54964438714199304</v>
+      </c>
+    </row>
+    <row r="69" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A69">
+        <v>68</v>
+      </c>
+      <c r="B69">
+        <v>50</v>
+      </c>
+      <c r="C69">
+        <v>26.8666666666666</v>
+      </c>
+      <c r="D69">
+        <v>68</v>
+      </c>
+      <c r="E69">
+        <v>0.83333733321036696</v>
+      </c>
+      <c r="F69">
+        <v>0.83468283769791496</v>
+      </c>
+      <c r="G69">
+        <v>68</v>
+      </c>
+      <c r="H69">
+        <v>1.80719191284298E-2</v>
+      </c>
+      <c r="I69">
+        <v>1.0170418752764599E-2</v>
+      </c>
+      <c r="J69">
+        <v>68</v>
+      </c>
+      <c r="K69">
+        <v>0.57899113104956001</v>
+      </c>
+      <c r="L69">
+        <v>0.54721221855914803</v>
+      </c>
+    </row>
+    <row r="70" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A70">
+        <v>69</v>
+      </c>
+      <c r="B70">
+        <v>49.7</v>
+      </c>
+      <c r="C70">
+        <v>26.3333333333333</v>
+      </c>
+      <c r="D70">
+        <v>69</v>
+      </c>
+      <c r="E70">
+        <v>0.83340637912266802</v>
+      </c>
+      <c r="F70">
+        <v>0.83473400643054396</v>
+      </c>
+      <c r="G70">
+        <v>69</v>
+      </c>
+      <c r="H70">
+        <v>1.7957824332433502E-2</v>
+      </c>
+      <c r="I70">
+        <v>1.0049070616387001E-2</v>
+      </c>
+      <c r="J70">
+        <v>69</v>
+      </c>
+      <c r="K70">
+        <v>0.57599198680548103</v>
+      </c>
+      <c r="L70">
+        <v>0.54483784949371905</v>
+      </c>
+    </row>
+    <row r="71" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A71">
+        <v>70</v>
+      </c>
+      <c r="B71">
+        <v>49.7</v>
+      </c>
+      <c r="C71">
+        <v>26.3333333333333</v>
+      </c>
+      <c r="D71">
+        <v>70</v>
+      </c>
+      <c r="E71">
+        <v>0.83340637912266802</v>
+      </c>
+      <c r="F71">
+        <v>0.83473400643054396</v>
+      </c>
+      <c r="G71">
+        <v>70</v>
+      </c>
+      <c r="H71">
+        <v>1.7957824332433502E-2</v>
+      </c>
+      <c r="I71">
+        <v>1.0049070616387001E-2</v>
+      </c>
+      <c r="J71">
+        <v>70</v>
+      </c>
+      <c r="K71">
+        <v>0.57599198680548103</v>
+      </c>
+      <c r="L71">
+        <v>0.54483784949371905</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="J1:K1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>